<commit_message>
PRIM: refresh run artifacts for futures, scenario discovery and dvc.lock
Regenerated PRIM pipeline outputs: per-future inputs/outputs and pickles
for Scenario1_1..20, base future executables (Scenario1_0, datasets 0),
aggregated futures parquets, scenario discovery files (t3b_sdiscovery),
control workbook and updated dvc.lock hashes.
</commit_message>
<xml_diff>
--- a/src/workflow/4_PRIM/t3b_sdiscovery/Units.xlsx
+++ b/src/workflow/4_PRIM/t3b_sdiscovery/Units.xlsx
@@ -809,9 +809,10 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F74FB0E003A88C4B9D9793633BA4B356" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="47be61afb57dbdcdac73424092eefa1c">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0d55314f-45f1-40c9-9fce-63556e193d03" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2e59f5c7e704c6a619606efe0cdd9ac5" ns2:_="">
-    <xsd:import namespace="0d55314f-45f1-40c9-9fce-63556e193d03"/>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101004DA328C4E73E6444AD0EEE0F2F633553" ma:contentTypeVersion="12" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="14698b2b587991840b26c8f9a5806477">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="0b4b13fe-0218-45f0-9474-10fbfc8ffc07" xmlns:ns3="91aae848-11ce-4a29-86ed-f19c4bd1a778" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bbde81f19d0bba47ecbb8881f798f31e" ns2:_="" ns3:_="">
+    <xsd:import namespace="0b4b13fe-0218-45f0-9474-10fbfc8ffc07"/>
+    <xsd:import namespace="91aae848-11ce-4a29-86ed-f19c4bd1a778"/>
     <xsd:element name="properties">
       <xsd:complexType>
         <xsd:sequence>
@@ -821,14 +822,14 @@
                 <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -836,7 +837,7 @@
       </xsd:complexType>
     </xsd:element>
   </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0d55314f-45f1-40c9-9fce-63556e193d03" elementFormDefault="qualified">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="0b4b13fe-0218-45f0-9474-10fbfc8ffc07" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
@@ -854,49 +855,59 @@
         <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+    <xsd:element name="MediaServiceDateTaken" ma:index="11" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="71f7bd95-1200-4052-9a4e-dfdf006e181b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="MediaServiceGenerationTime" ma:index="12" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="13" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="14" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="15" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="71f7bd95-1200-4052-9a4e-dfdf006e181b" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
         </xsd:sequence>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="14" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="15" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+    <xsd:element name="MediaServiceOCR" ma:index="19" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
         </xsd:restriction>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="16" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="17" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="18" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="91aae848-11ce-4a29-86ed-f19c4bd1a778" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="18" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{265747d2-66b6-4563-8f7b-1a6180f74c1f}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="91aae848-11ce-4a29-86ed-f19c4bd1a778">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
     </xsd:element>
   </xsd:schema>
   <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
@@ -1001,9 +1012,10 @@
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0d55314f-45f1-40c9-9fce-63556e193d03">
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="0b4b13fe-0218-45f0-9474-10fbfc8ffc07">
       <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="91aae848-11ce-4a29-86ed-f19c4bd1a778" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
 </file>
@@ -1018,21 +1030,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AEFFD235-2FD9-45D9-BE4E-E906BFFC66BB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="0d55314f-45f1-40c9-9fce-63556e193d03"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{11504A77-5DA9-4A99-A8D6-59CB29F18236}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>